<commit_message>
Fix shipping upload product name matching
</commit_message>
<xml_diff>
--- a/public/shipping-template.xlsx
+++ b/public/shipping-template.xlsx
@@ -1,47 +1,104 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="배송대행" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="배송대행" state="visible" r:id="rId4"/>
   </sheets>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="25">
+  <si>
+    <t>배송대행 업로드 양식</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>CJ대한통운 기준 · 쿠팡/토스 통일 양식</t>
+  </si>
+  <si>
+    <t>업로드 정보</t>
+  </si>
+  <si>
+    <t>상호</t>
+  </si>
+  <si>
+    <t>(예: ABC상사)</t>
+  </si>
+  <si>
+    <t>담당자 연락처</t>
+  </si>
+  <si>
+    <t>010-0000-0000</t>
+  </si>
+  <si>
+    <t>요청사항</t>
+  </si>
+  <si>
+    <t>(공통 메모, 선택)</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>받는사람</t>
+  </si>
+  <si>
+    <t>연락처</t>
+  </si>
+  <si>
+    <t>주소</t>
+  </si>
+  <si>
+    <t>상품명</t>
+  </si>
+  <si>
+    <t>옵션</t>
+  </si>
+  <si>
+    <t>수량</t>
+  </si>
+  <si>
+    <t>메모</t>
+  </si>
+  <si>
+    <t>송장번호</t>
+  </si>
+  <si>
+    <t>예시 홍길동</t>
+  </si>
+  <si>
+    <t>010-1234-5678</t>
+  </si>
+  <si>
+    <t>서울시 강남구 ...</t>
+  </si>
+  <si>
+    <t>스니커즈</t>
+  </si>
+  <si>
+    <t>270</t>
+  </si>
+  <si>
+    <t>문 앞에 두세요</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -65,13 +122,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,255 +461,255 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I10"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="5.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="24.83203125" customWidth="1"/>
-    <col min="7" max="7" width="6.83203125" customWidth="1"/>
-    <col min="8" max="8" width="20.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="36" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="24" customWidth="1"/>
+    <col min="7" max="7" width="6" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>배송대행 업로드 양식</v>
-      </c>
-      <c r="B1" t="str">
-        <v/>
-      </c>
-      <c r="C1" t="str">
-        <v/>
-      </c>
-      <c r="D1" t="str">
-        <v/>
-      </c>
-      <c r="E1" t="str">
-        <v/>
-      </c>
-      <c r="F1" t="str">
-        <v/>
-      </c>
-      <c r="G1" t="str">
-        <v/>
-      </c>
-      <c r="H1" t="str">
-        <v/>
-      </c>
-      <c r="I1" t="str">
-        <v/>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" t="s">
+        <v>1</v>
+      </c>
+      <c r="I1" t="s">
+        <v>1</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>CJ대한통운 기준 · 쿠팡/스스 통일 양식</v>
-      </c>
-      <c r="B2" t="str">
-        <v/>
-      </c>
-      <c r="C2" t="str">
-        <v/>
-      </c>
-      <c r="D2" t="str">
-        <v/>
-      </c>
-      <c r="E2" t="str">
-        <v/>
-      </c>
-      <c r="F2" t="str">
-        <v/>
-      </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
-      <c r="H2" t="str">
-        <v/>
-      </c>
-      <c r="I2" t="str">
-        <v/>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" t="s">
+        <v>1</v>
+      </c>
+      <c r="H2" t="s">
+        <v>1</v>
+      </c>
+      <c r="I2" t="s">
+        <v>1</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>업로더 정보</v>
-      </c>
-      <c r="B4" t="str">
-        <v/>
-      </c>
-      <c r="C4" t="str">
-        <v/>
-      </c>
-      <c r="D4" t="str">
-        <v/>
-      </c>
-      <c r="E4" t="str">
-        <v/>
-      </c>
-      <c r="F4" t="str">
-        <v/>
-      </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
-      <c r="H4" t="str">
-        <v/>
-      </c>
-      <c r="I4" t="str">
-        <v/>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
+        <v>1</v>
+      </c>
+      <c r="F4" t="s">
+        <v>1</v>
+      </c>
+      <c r="G4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H4" t="s">
+        <v>1</v>
+      </c>
+      <c r="I4" t="s">
+        <v>1</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>상호</v>
-      </c>
-      <c r="B5" t="str">
-        <v>(예: ABC상사)</v>
-      </c>
-      <c r="C5" t="str">
-        <v>담당자 연락처</v>
-      </c>
-      <c r="D5" t="str">
-        <v>010-0000-0000</v>
-      </c>
-      <c r="E5" t="str">
-        <v/>
-      </c>
-      <c r="F5" t="str">
-        <v/>
-      </c>
-      <c r="G5" t="str">
-        <v/>
-      </c>
-      <c r="H5" t="str">
-        <v/>
-      </c>
-      <c r="I5" t="str">
-        <v/>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" t="s">
+        <v>1</v>
+      </c>
+      <c r="F5" t="s">
+        <v>1</v>
+      </c>
+      <c r="G5" t="s">
+        <v>1</v>
+      </c>
+      <c r="H5" t="s">
+        <v>1</v>
+      </c>
+      <c r="I5" t="s">
+        <v>1</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>요청사항</v>
-      </c>
-      <c r="B6" t="str">
-        <v>(공통 메모, 선택)</v>
-      </c>
-      <c r="C6" t="str">
-        <v/>
-      </c>
-      <c r="D6" t="str">
-        <v/>
-      </c>
-      <c r="E6" t="str">
-        <v/>
-      </c>
-      <c r="F6" t="str">
-        <v/>
-      </c>
-      <c r="G6" t="str">
-        <v/>
-      </c>
-      <c r="H6" t="str">
-        <v/>
-      </c>
-      <c r="I6" t="str">
-        <v/>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>1</v>
+      </c>
+      <c r="E6" t="s">
+        <v>1</v>
+      </c>
+      <c r="F6" t="s">
+        <v>1</v>
+      </c>
+      <c r="G6" t="s">
+        <v>1</v>
+      </c>
+      <c r="H6" t="s">
+        <v>1</v>
+      </c>
+      <c r="I6" t="s">
+        <v>1</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>No</v>
-      </c>
-      <c r="B8" t="str">
-        <v>받는사람*</v>
-      </c>
-      <c r="C8" t="str">
-        <v>연락처*</v>
-      </c>
-      <c r="D8" t="str">
-        <v>주소*</v>
-      </c>
-      <c r="E8" t="str">
-        <v>관리코드*</v>
-      </c>
-      <c r="F8" t="str">
-        <v>상품명/옵션</v>
-      </c>
-      <c r="G8" t="str">
-        <v>수량*</v>
-      </c>
-      <c r="H8" t="str">
-        <v>메모</v>
-      </c>
-      <c r="I8" t="str">
-        <v>송장번호</v>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" t="s">
+        <v>15</v>
+      </c>
+      <c r="G8" t="s">
+        <v>16</v>
+      </c>
+      <c r="H8" t="s">
+        <v>17</v>
+      </c>
+      <c r="I8" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1</v>
       </c>
-      <c r="B9" t="str">
-        <v>예시 홍길동</v>
-      </c>
-      <c r="C9" t="str">
-        <v>010-1234-5678</v>
-      </c>
-      <c r="D9" t="str">
-        <v>서울시 강남구 ...</v>
-      </c>
-      <c r="E9" t="str">
-        <v>SKR-001</v>
-      </c>
-      <c r="F9" t="str">
-        <v>스니커즈/270</v>
+      <c r="B9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" t="s">
+        <v>23</v>
       </c>
       <c r="G9">
         <v>1</v>
       </c>
-      <c r="H9" t="str">
-        <v>문 앞에 두어주세요</v>
-      </c>
-      <c r="I9" t="str">
-        <v/>
+      <c r="H9" t="s">
+        <v>24</v>
+      </c>
+      <c r="I9" t="s">
+        <v>1</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2</v>
       </c>
-      <c r="B10" t="str">
-        <v/>
-      </c>
-      <c r="C10" t="str">
-        <v/>
-      </c>
-      <c r="D10" t="str">
-        <v/>
-      </c>
-      <c r="E10" t="str">
-        <v/>
-      </c>
-      <c r="F10" t="str">
-        <v/>
-      </c>
-      <c r="G10" t="str">
-        <v/>
-      </c>
-      <c r="H10" t="str">
-        <v/>
-      </c>
-      <c r="I10" t="str">
-        <v/>
+      <c r="B10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D10" t="s">
+        <v>1</v>
+      </c>
+      <c r="E10" t="s">
+        <v>1</v>
+      </c>
+      <c r="F10" t="s">
+        <v>1</v>
+      </c>
+      <c r="G10" t="s">
+        <v>1</v>
+      </c>
+      <c r="H10" t="s">
+        <v>1</v>
+      </c>
+      <c r="I10" t="s">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I10"/>
-  </ignoredErrors>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix shipping upload product name matching (#6)
</commit_message>
<xml_diff>
--- a/public/shipping-template.xlsx
+++ b/public/shipping-template.xlsx
@@ -1,47 +1,104 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="배송대행" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="배송대행" state="visible" r:id="rId4"/>
   </sheets>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="25">
+  <si>
+    <t>배송대행 업로드 양식</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>CJ대한통운 기준 · 쿠팡/토스 통일 양식</t>
+  </si>
+  <si>
+    <t>업로드 정보</t>
+  </si>
+  <si>
+    <t>상호</t>
+  </si>
+  <si>
+    <t>(예: ABC상사)</t>
+  </si>
+  <si>
+    <t>담당자 연락처</t>
+  </si>
+  <si>
+    <t>010-0000-0000</t>
+  </si>
+  <si>
+    <t>요청사항</t>
+  </si>
+  <si>
+    <t>(공통 메모, 선택)</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>받는사람</t>
+  </si>
+  <si>
+    <t>연락처</t>
+  </si>
+  <si>
+    <t>주소</t>
+  </si>
+  <si>
+    <t>상품명</t>
+  </si>
+  <si>
+    <t>옵션</t>
+  </si>
+  <si>
+    <t>수량</t>
+  </si>
+  <si>
+    <t>메모</t>
+  </si>
+  <si>
+    <t>송장번호</t>
+  </si>
+  <si>
+    <t>예시 홍길동</t>
+  </si>
+  <si>
+    <t>010-1234-5678</t>
+  </si>
+  <si>
+    <t>서울시 강남구 ...</t>
+  </si>
+  <si>
+    <t>스니커즈</t>
+  </si>
+  <si>
+    <t>270</t>
+  </si>
+  <si>
+    <t>문 앞에 두세요</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -65,13 +122,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,255 +461,255 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I10"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="5.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="24.83203125" customWidth="1"/>
-    <col min="7" max="7" width="6.83203125" customWidth="1"/>
-    <col min="8" max="8" width="20.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="36" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="24" customWidth="1"/>
+    <col min="7" max="7" width="6" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>배송대행 업로드 양식</v>
-      </c>
-      <c r="B1" t="str">
-        <v/>
-      </c>
-      <c r="C1" t="str">
-        <v/>
-      </c>
-      <c r="D1" t="str">
-        <v/>
-      </c>
-      <c r="E1" t="str">
-        <v/>
-      </c>
-      <c r="F1" t="str">
-        <v/>
-      </c>
-      <c r="G1" t="str">
-        <v/>
-      </c>
-      <c r="H1" t="str">
-        <v/>
-      </c>
-      <c r="I1" t="str">
-        <v/>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" t="s">
+        <v>1</v>
+      </c>
+      <c r="I1" t="s">
+        <v>1</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>CJ대한통운 기준 · 쿠팡/스스 통일 양식</v>
-      </c>
-      <c r="B2" t="str">
-        <v/>
-      </c>
-      <c r="C2" t="str">
-        <v/>
-      </c>
-      <c r="D2" t="str">
-        <v/>
-      </c>
-      <c r="E2" t="str">
-        <v/>
-      </c>
-      <c r="F2" t="str">
-        <v/>
-      </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
-      <c r="H2" t="str">
-        <v/>
-      </c>
-      <c r="I2" t="str">
-        <v/>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" t="s">
+        <v>1</v>
+      </c>
+      <c r="H2" t="s">
+        <v>1</v>
+      </c>
+      <c r="I2" t="s">
+        <v>1</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>업로더 정보</v>
-      </c>
-      <c r="B4" t="str">
-        <v/>
-      </c>
-      <c r="C4" t="str">
-        <v/>
-      </c>
-      <c r="D4" t="str">
-        <v/>
-      </c>
-      <c r="E4" t="str">
-        <v/>
-      </c>
-      <c r="F4" t="str">
-        <v/>
-      </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
-      <c r="H4" t="str">
-        <v/>
-      </c>
-      <c r="I4" t="str">
-        <v/>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
+        <v>1</v>
+      </c>
+      <c r="F4" t="s">
+        <v>1</v>
+      </c>
+      <c r="G4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H4" t="s">
+        <v>1</v>
+      </c>
+      <c r="I4" t="s">
+        <v>1</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>상호</v>
-      </c>
-      <c r="B5" t="str">
-        <v>(예: ABC상사)</v>
-      </c>
-      <c r="C5" t="str">
-        <v>담당자 연락처</v>
-      </c>
-      <c r="D5" t="str">
-        <v>010-0000-0000</v>
-      </c>
-      <c r="E5" t="str">
-        <v/>
-      </c>
-      <c r="F5" t="str">
-        <v/>
-      </c>
-      <c r="G5" t="str">
-        <v/>
-      </c>
-      <c r="H5" t="str">
-        <v/>
-      </c>
-      <c r="I5" t="str">
-        <v/>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" t="s">
+        <v>1</v>
+      </c>
+      <c r="F5" t="s">
+        <v>1</v>
+      </c>
+      <c r="G5" t="s">
+        <v>1</v>
+      </c>
+      <c r="H5" t="s">
+        <v>1</v>
+      </c>
+      <c r="I5" t="s">
+        <v>1</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>요청사항</v>
-      </c>
-      <c r="B6" t="str">
-        <v>(공통 메모, 선택)</v>
-      </c>
-      <c r="C6" t="str">
-        <v/>
-      </c>
-      <c r="D6" t="str">
-        <v/>
-      </c>
-      <c r="E6" t="str">
-        <v/>
-      </c>
-      <c r="F6" t="str">
-        <v/>
-      </c>
-      <c r="G6" t="str">
-        <v/>
-      </c>
-      <c r="H6" t="str">
-        <v/>
-      </c>
-      <c r="I6" t="str">
-        <v/>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>1</v>
+      </c>
+      <c r="E6" t="s">
+        <v>1</v>
+      </c>
+      <c r="F6" t="s">
+        <v>1</v>
+      </c>
+      <c r="G6" t="s">
+        <v>1</v>
+      </c>
+      <c r="H6" t="s">
+        <v>1</v>
+      </c>
+      <c r="I6" t="s">
+        <v>1</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>No</v>
-      </c>
-      <c r="B8" t="str">
-        <v>받는사람*</v>
-      </c>
-      <c r="C8" t="str">
-        <v>연락처*</v>
-      </c>
-      <c r="D8" t="str">
-        <v>주소*</v>
-      </c>
-      <c r="E8" t="str">
-        <v>관리코드*</v>
-      </c>
-      <c r="F8" t="str">
-        <v>상품명/옵션</v>
-      </c>
-      <c r="G8" t="str">
-        <v>수량*</v>
-      </c>
-      <c r="H8" t="str">
-        <v>메모</v>
-      </c>
-      <c r="I8" t="str">
-        <v>송장번호</v>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" t="s">
+        <v>15</v>
+      </c>
+      <c r="G8" t="s">
+        <v>16</v>
+      </c>
+      <c r="H8" t="s">
+        <v>17</v>
+      </c>
+      <c r="I8" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1</v>
       </c>
-      <c r="B9" t="str">
-        <v>예시 홍길동</v>
-      </c>
-      <c r="C9" t="str">
-        <v>010-1234-5678</v>
-      </c>
-      <c r="D9" t="str">
-        <v>서울시 강남구 ...</v>
-      </c>
-      <c r="E9" t="str">
-        <v>SKR-001</v>
-      </c>
-      <c r="F9" t="str">
-        <v>스니커즈/270</v>
+      <c r="B9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" t="s">
+        <v>23</v>
       </c>
       <c r="G9">
         <v>1</v>
       </c>
-      <c r="H9" t="str">
-        <v>문 앞에 두어주세요</v>
-      </c>
-      <c r="I9" t="str">
-        <v/>
+      <c r="H9" t="s">
+        <v>24</v>
+      </c>
+      <c r="I9" t="s">
+        <v>1</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2</v>
       </c>
-      <c r="B10" t="str">
-        <v/>
-      </c>
-      <c r="C10" t="str">
-        <v/>
-      </c>
-      <c r="D10" t="str">
-        <v/>
-      </c>
-      <c r="E10" t="str">
-        <v/>
-      </c>
-      <c r="F10" t="str">
-        <v/>
-      </c>
-      <c r="G10" t="str">
-        <v/>
-      </c>
-      <c r="H10" t="str">
-        <v/>
-      </c>
-      <c r="I10" t="str">
-        <v/>
+      <c r="B10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D10" t="s">
+        <v>1</v>
+      </c>
+      <c r="E10" t="s">
+        <v>1</v>
+      </c>
+      <c r="F10" t="s">
+        <v>1</v>
+      </c>
+      <c r="G10" t="s">
+        <v>1</v>
+      </c>
+      <c r="H10" t="s">
+        <v>1</v>
+      </c>
+      <c r="I10" t="s">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I10"/>
-  </ignoredErrors>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: finalize shipping upload follow-ups
</commit_message>
<xml_diff>
--- a/public/shipping-template.xlsx
+++ b/public/shipping-template.xlsx
@@ -3,9 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
-  <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
-  </bookViews>
   <sheets>
     <sheet sheetId="1" name="배송대행" state="visible" r:id="rId4"/>
   </sheets>
@@ -14,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="24">
   <si>
     <t>배송대행 업로드 양식</t>
   </si>
@@ -22,7 +19,7 @@
     <t/>
   </si>
   <si>
-    <t>CJ대한통운 기준 · 쿠팡/토스 통일 양식</t>
+    <t>CJ대한통운 기준 통합 양식</t>
   </si>
   <si>
     <t>업로드 정보</t>
@@ -31,13 +28,13 @@
     <t>상호</t>
   </si>
   <si>
-    <t>제이컴퍼니</t>
+    <t>(예: ABC상사)</t>
   </si>
   <si>
     <t>담당자 연락처</t>
   </si>
   <si>
-    <t>010-1234-5678</t>
+    <t>010-0000-0000</t>
   </si>
   <si>
     <t>요청사항</t>
@@ -92,7 +89,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -100,28 +97,16 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <color theme="1"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="맑은 고딕"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFDDDDDD"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -129,32 +114,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -495,15 +461,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I1008"/>
-  <sheetFormatPr defaultRowHeight="17.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.4" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="36" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="24" customWidth="1"/>
-    <col min="7" max="7" width="6" customWidth="1"/>
+    <col min="7" max="7" width="8" customWidth="1"/>
     <col min="8" max="8" width="20" customWidth="1"/>
     <col min="9" max="9" width="16" style="1" customWidth="1"/>
   </cols>
@@ -657,25 +623,25 @@
       <c r="A8" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" t="s">
         <v>13</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" t="s">
         <v>14</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" t="s">
         <v>15</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="G8" t="s">
         <v>16</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" t="s">
         <v>17</v>
       </c>
       <c r="I8" s="1" t="s">
@@ -698,13 +664,16 @@
       <c r="E9" t="s">
         <v>22</v>
       </c>
+      <c r="F9" t="s">
+        <v>1</v>
+      </c>
       <c r="G9">
         <v>1</v>
       </c>
       <c r="H9" t="s">
         <v>23</v>
       </c>
-      <c r="I9" s="3">
+      <c r="I9" s="1">
         <v>521853092894</v>
       </c>
     </row>
@@ -3733,6 +3702,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>